<commit_message>
struct > class 구조변경작업.
</commit_message>
<xml_diff>
--- a/ExcelToJSONConverter/excel/item.xlsx
+++ b/ExcelToJSONConverter/excel/item.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4971F4E1-006C-4B8B-A926-B0354DA9B9EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE271B3F-F234-4BC9-BDF7-4C7489D34F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1395" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="1395" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="151">
   <si>
     <t>string</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -492,13 +492,22 @@
   </si>
   <si>
     <t>{"life_steal":1,"move_speed":1}</t>
+  </si>
+  <si>
+    <t>Normal_Gatcha_Ticket</t>
+  </si>
+  <si>
+    <t>Rare_Gatcha_Ticket</t>
+  </si>
+  <si>
+    <t>Tournament_Point</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -532,6 +541,12 @@
     <font>
       <b/>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -672,7 +687,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -681,9 +696,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -720,6 +732,21 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1059,7 +1086,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.25" bestFit="1" customWidth="1"/>
@@ -1081,7 +1108,7 @@
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G2" t="s">
@@ -1099,9 +1126,10 @@
         <v>2</v>
       </c>
       <c r="D3">
+        <f>D2+1</f>
         <v>2</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="G3" t="s">
@@ -1119,9 +1147,10 @@
         <v>3</v>
       </c>
       <c r="D4">
+        <f t="shared" ref="D4:D20" si="0">D3+1</f>
         <v>3</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G4" t="s">
@@ -1139,9 +1168,10 @@
         <v>4</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>20</v>
       </c>
       <c r="G5" t="s">
@@ -1159,9 +1189,10 @@
         <v>5</v>
       </c>
       <c r="D6">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>21</v>
       </c>
       <c r="G6" t="s">
@@ -1179,90 +1210,128 @@
         <v>6</v>
       </c>
       <c r="D7">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D8">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D9">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D10">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="D11">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="D12">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D13">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D14">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D15">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D16">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="17" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D17">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D18">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="E18" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="19" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D19">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="E19" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="20" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D20">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="E20" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1274,11 +1343,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.625" style="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.375" bestFit="1" customWidth="1"/>
   </cols>
@@ -1287,7 +1356,7 @@
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="17" t="s">
         <v>33</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1301,7 +1370,7 @@
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="18" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="1"/>
@@ -1310,274 +1379,325 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
+      <c r="A3" s="15">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="str">
+      <c r="B3" s="16" t="str">
         <f>VLOOKUP(A3,Overview!D2:E34,2,FALSE)</f>
         <v>rice</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="15">
         <f>VLOOKUP(C3,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
+      <c r="A4" s="15">
         <f>A3+1</f>
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="str">
+      <c r="B4" s="16" t="str">
         <f>VLOOKUP(A4,Overview!D3:E35,2,FALSE)</f>
         <v>gold</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="15">
         <f>VLOOKUP(C4,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
-        <f t="shared" ref="A5:A18" si="0">A4+1</f>
+      <c r="A5" s="15">
+        <f t="shared" ref="A5:A21" si="0">A4+1</f>
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="16" t="str">
         <f>VLOOKUP(A5,Overview!D4:E36,2,FALSE)</f>
         <v>time_stone</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="15">
         <f>VLOOKUP(C5,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
+      <c r="A6" s="15">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="16" t="str">
         <f>VLOOKUP(A6,Overview!D5:E37,2,FALSE)</f>
         <v>bundle_normal</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="15">
         <f>VLOOKUP(C6,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+      <c r="A7" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="str">
+      <c r="B7" s="16" t="str">
         <f>VLOOKUP(A7,Overview!D6:E38,2,FALSE)</f>
         <v>bundle_elite</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="15">
         <f>VLOOKUP(C7,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
+      <c r="A8" s="15">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="str">
+      <c r="B8" s="16" t="str">
         <f>VLOOKUP(A8,Overview!D7:E39,2,FALSE)</f>
         <v>bundle_general</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="15">
         <f>VLOOKUP(C8,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
+      <c r="A9" s="15">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="str">
+      <c r="B9" s="16" t="str">
         <f>VLOOKUP(A9,Overview!D8:E40,2,FALSE)</f>
         <v>bundle_hero</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="15">
         <f>VLOOKUP(C9,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="3">
+      <c r="A10" s="15">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B10" s="4" t="str">
+      <c r="B10" s="16" t="str">
         <f>VLOOKUP(A10,Overview!D9:E41,2,FALSE)</f>
         <v>bundle_legend</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="15">
         <f>VLOOKUP(C10,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="3">
+      <c r="A11" s="15">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="str">
+      <c r="B11" s="16" t="str">
         <f>VLOOKUP(A11,Overview!D10:E42,2,FALSE)</f>
         <v>public_soul_stone</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="15">
         <f>VLOOKUP(C11,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
+      <c r="A12" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B12" s="4" t="str">
+      <c r="B12" s="16" t="str">
         <f>VLOOKUP(A12,Overview!D11:E43,2,FALSE)</f>
         <v>class_soul_stone</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="15">
         <f>VLOOKUP(C12,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="3">
+      <c r="A13" s="15">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B13" s="4" t="str">
+      <c r="B13" s="16" t="str">
         <f>VLOOKUP(A13,Overview!D12:E44,2,FALSE)</f>
         <v>dedicated_soul_stone</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="15">
         <f>VLOOKUP(C13,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="3">
+    <row r="14" spans="1:4" ht="28.5" x14ac:dyDescent="0.3">
+      <c r="A14" s="15">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B14" s="4" t="str">
+      <c r="B14" s="16" t="str">
         <f>VLOOKUP(A14,Overview!D13:E45,2,FALSE)</f>
         <v>class_soul_stone_random_box</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="15">
         <f>VLOOKUP(C14,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="3">
+    <row r="15" spans="1:4" ht="28.5" x14ac:dyDescent="0.3">
+      <c r="A15" s="15">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B15" s="4" t="str">
+      <c r="B15" s="16" t="str">
         <f>VLOOKUP(A15,Overview!D14:E46,2,FALSE)</f>
         <v>dedicated_soul_stone_random_box</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="15">
         <f>VLOOKUP(C15,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="3">
+      <c r="A16" s="15">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="B16" s="4" t="str">
+      <c r="B16" s="16" t="str">
         <f>VLOOKUP(A16,Overview!D15:E47,2,FALSE)</f>
         <v>treasure</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="15">
         <f>VLOOKUP(C16,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="3">
+      <c r="A17" s="15">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="B17" s="4" t="str">
+      <c r="B17" s="16" t="str">
         <f>VLOOKUP(A17,Overview!D16:E48,2,FALSE)</f>
         <v>treasure_piece</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="15">
         <f>VLOOKUP(C17,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="3">
+    <row r="18" spans="1:4" ht="28.5" x14ac:dyDescent="0.3">
+      <c r="A18" s="15">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B18" s="4" t="str">
+      <c r="B18" s="16" t="str">
         <f>VLOOKUP(A18,Overview!D17:E49,2,FALSE)</f>
         <v>treasure_piece_random_box</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="15">
         <f>VLOOKUP(C18,Overview!$A$2:$B$7,2,FALSE)</f>
         <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="15">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="B19" s="16" t="str">
+        <f>VLOOKUP(A19,Overview!D18:E50,2,FALSE)</f>
+        <v>Normal_Gatcha_Ticket</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="15">
+        <f>VLOOKUP(C19,Overview!$A$2:$B$7,2,FALSE)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="15">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="B20" s="16" t="str">
+        <f>VLOOKUP(A20,Overview!D19:E51,2,FALSE)</f>
+        <v>Rare_Gatcha_Ticket</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="15">
+        <f>VLOOKUP(C20,Overview!$A$2:$B$7,2,FALSE)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="15">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="B21" s="16" t="str">
+        <f>VLOOKUP(A21,Overview!D20:E52,2,FALSE)</f>
+        <v>Tournament_Point</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="15">
+        <f>VLOOKUP(C21,Overview!$A$2:$B$7,2,FALSE)</f>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1601,907 +1721,907 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <f>VLOOKUP(C3,Overview!$G$2:$H$6,2,)</f>
         <v>0</v>
       </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="10">
+      <c r="E3" s="13"/>
+      <c r="F3" s="9">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <f>VLOOKUP(C4,Overview!$G$2:$H$6,2,)</f>
         <v>0</v>
       </c>
-      <c r="E4" s="15"/>
-      <c r="F4" s="11">
+      <c r="E4" s="14"/>
+      <c r="F4" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <f>VLOOKUP(C5,Overview!$G$2:$H$6,2,)</f>
         <v>0</v>
       </c>
-      <c r="E5" s="15"/>
-      <c r="F5" s="11">
+      <c r="E5" s="14"/>
+      <c r="F5" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <f>VLOOKUP(C6,Overview!$G$2:$H$6,2,)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="15"/>
-      <c r="F6" s="11">
+      <c r="E6" s="14"/>
+      <c r="F6" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <f>VLOOKUP(C7,Overview!$G$2:$H$6,2,)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="15"/>
-      <c r="F7" s="11">
+      <c r="E7" s="14"/>
+      <c r="F7" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="9">
         <f>VLOOKUP(C8,Overview!$G$2:$H$6,2,)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="15"/>
-      <c r="F8" s="11">
+      <c r="E8" s="14"/>
+      <c r="F8" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="9">
         <f>VLOOKUP(C9,Overview!$G$2:$H$6,2,)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="15"/>
-      <c r="F9" s="11">
+      <c r="E9" s="14"/>
+      <c r="F9" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="9">
         <f>VLOOKUP(C10,Overview!$G$2:$H$6,2,)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="15"/>
-      <c r="F10" s="11">
+      <c r="E10" s="14"/>
+      <c r="F10" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <f>VLOOKUP(C11,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="9">
         <f>VLOOKUP(C12,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <f>VLOOKUP(C13,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E13" s="15"/>
-      <c r="F13" s="11">
+      <c r="E13" s="14"/>
+      <c r="F13" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <f>VLOOKUP(C14,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E14" s="15"/>
-      <c r="F14" s="11">
+      <c r="E14" s="14"/>
+      <c r="F14" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="9">
         <f>VLOOKUP(C15,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E15" s="15"/>
-      <c r="F15" s="11">
+      <c r="E15" s="14"/>
+      <c r="F15" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="9">
         <f>VLOOKUP(C16,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E16" s="15"/>
-      <c r="F16" s="11">
+      <c r="E16" s="14"/>
+      <c r="F16" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="9">
         <f>VLOOKUP(C17,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E17" s="15"/>
-      <c r="F17" s="11">
+      <c r="E17" s="14"/>
+      <c r="F17" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <f>VLOOKUP(C18,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E18" s="15"/>
-      <c r="F18" s="11">
+      <c r="E18" s="14"/>
+      <c r="F18" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="9">
         <f>VLOOKUP(C19,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E19" s="15"/>
-      <c r="F19" s="11">
+      <c r="E19" s="14"/>
+      <c r="F19" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <f>VLOOKUP(C20,Overview!$G$2:$H$6,2,)</f>
         <v>1</v>
       </c>
-      <c r="E20" s="15"/>
-      <c r="F20" s="11">
+      <c r="E20" s="14"/>
+      <c r="F20" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="9">
         <f>VLOOKUP(C21,Overview!$G$2:$H$6,2,)</f>
         <v>2</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D22" s="10">
+      <c r="D22" s="9">
         <f>VLOOKUP(C22,Overview!$G$2:$H$6,2,)</f>
         <v>2</v>
       </c>
-      <c r="E22" s="15"/>
-      <c r="F22" s="11">
+      <c r="E22" s="14"/>
+      <c r="F22" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="9">
         <f>VLOOKUP(C23,Overview!$G$2:$H$6,2,)</f>
         <v>2</v>
       </c>
-      <c r="E23" s="15"/>
-      <c r="F23" s="11">
+      <c r="E23" s="14"/>
+      <c r="F23" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="9">
         <f>VLOOKUP(C24,Overview!$G$2:$H$6,2,)</f>
         <v>2</v>
       </c>
-      <c r="E24" s="15"/>
-      <c r="F24" s="11">
+      <c r="E24" s="14"/>
+      <c r="F24" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="9">
         <f>VLOOKUP(C25,Overview!$G$2:$H$6,2,)</f>
         <v>2</v>
       </c>
-      <c r="E25" s="15"/>
-      <c r="F25" s="11">
+      <c r="E25" s="14"/>
+      <c r="F25" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <f>VLOOKUP(C26,Overview!$G$2:$H$6,2,)</f>
         <v>2</v>
       </c>
-      <c r="E26" s="15"/>
-      <c r="F26" s="11">
+      <c r="E26" s="14"/>
+      <c r="F26" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="9">
         <f>VLOOKUP(C27,Overview!$G$2:$H$6,2,)</f>
         <v>2</v>
       </c>
-      <c r="E27" s="15"/>
-      <c r="F27" s="11">
+      <c r="E27" s="14"/>
+      <c r="F27" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D28" s="10">
+      <c r="D28" s="9">
         <f>VLOOKUP(C28,Overview!$G$2:$H$6,2,)</f>
         <v>2</v>
       </c>
-      <c r="E28" s="15"/>
-      <c r="F28" s="11">
+      <c r="E28" s="14"/>
+      <c r="F28" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D29" s="9">
         <f>VLOOKUP(C29,Overview!$G$2:$H$6,2,)</f>
         <v>2</v>
       </c>
-      <c r="E29" s="15"/>
-      <c r="F29" s="11">
+      <c r="E29" s="14"/>
+      <c r="F29" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="9">
         <f>VLOOKUP(C30,Overview!$G$2:$H$6,2,)</f>
         <v>3</v>
       </c>
-      <c r="E30" s="11" t="s">
+      <c r="E30" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="9">
         <f>VLOOKUP(C31,Overview!$G$2:$H$6,2,)</f>
         <v>3</v>
       </c>
-      <c r="E31" s="15"/>
-      <c r="F31" s="11">
+      <c r="E31" s="14"/>
+      <c r="F31" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D32" s="10">
+      <c r="D32" s="9">
         <f>VLOOKUP(C32,Overview!$G$2:$H$6,2,)</f>
         <v>3</v>
       </c>
-      <c r="E32" s="15"/>
-      <c r="F32" s="11">
+      <c r="E32" s="14"/>
+      <c r="F32" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="C33" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D33" s="10">
+      <c r="D33" s="9">
         <f>VLOOKUP(C33,Overview!$G$2:$H$6,2,)</f>
         <v>3</v>
       </c>
-      <c r="E33" s="15"/>
-      <c r="F33" s="11">
+      <c r="E33" s="14"/>
+      <c r="F33" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="11" t="s">
+      <c r="A34" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D34" s="10">
+      <c r="D34" s="9">
         <f>VLOOKUP(C34,Overview!$G$2:$H$6,2,)</f>
         <v>3</v>
       </c>
-      <c r="E34" s="15"/>
-      <c r="F34" s="11">
+      <c r="E34" s="14"/>
+      <c r="F34" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="11" t="s">
+      <c r="A35" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="C35" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D35" s="10">
+      <c r="D35" s="9">
         <f>VLOOKUP(C35,Overview!$G$2:$H$6,2,)</f>
         <v>3</v>
       </c>
-      <c r="E35" s="15"/>
-      <c r="F35" s="11">
+      <c r="E35" s="14"/>
+      <c r="F35" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D36" s="10">
+      <c r="D36" s="9">
         <f>VLOOKUP(C36,Overview!$G$2:$H$6,2,)</f>
         <v>3</v>
       </c>
-      <c r="E36" s="15"/>
-      <c r="F36" s="11">
+      <c r="E36" s="14"/>
+      <c r="F36" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="11" t="s">
+      <c r="A37" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D37" s="10">
+      <c r="D37" s="9">
         <f>VLOOKUP(C37,Overview!$G$2:$H$6,2,)</f>
         <v>3</v>
       </c>
-      <c r="E37" s="15"/>
-      <c r="F37" s="11">
+      <c r="E37" s="14"/>
+      <c r="F37" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="11" t="s">
+      <c r="A38" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="9">
         <f>VLOOKUP(C38,Overview!$G$2:$H$6,2,)</f>
         <v>3</v>
       </c>
-      <c r="E38" s="15"/>
-      <c r="F38" s="11">
+      <c r="E38" s="14"/>
+      <c r="F38" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="11" t="s">
+      <c r="A39" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="C39" s="11" t="s">
+      <c r="C39" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D39" s="10">
+      <c r="D39" s="9">
         <f>VLOOKUP(C39,Overview!$G$2:$H$6,2,)</f>
         <v>4</v>
       </c>
-      <c r="E39" s="11" t="s">
+      <c r="E39" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="F39" s="11">
+      <c r="F39" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="11" t="s">
+      <c r="A40" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D40" s="10">
+      <c r="D40" s="9">
         <f>VLOOKUP(C40,Overview!$G$2:$H$6,2,)</f>
         <v>4</v>
       </c>
-      <c r="E40" s="15"/>
-      <c r="F40" s="11">
+      <c r="E40" s="14"/>
+      <c r="F40" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="11" t="s">
+      <c r="A41" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="C41" s="11" t="s">
+      <c r="C41" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D41" s="10">
+      <c r="D41" s="9">
         <f>VLOOKUP(C41,Overview!$G$2:$H$6,2,)</f>
         <v>4</v>
       </c>
-      <c r="E41" s="15"/>
-      <c r="F41" s="11">
+      <c r="E41" s="14"/>
+      <c r="F41" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="11" t="s">
+      <c r="A42" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D42" s="9">
         <f>VLOOKUP(C42,Overview!$G$2:$H$6,2,)</f>
         <v>4</v>
       </c>
-      <c r="E42" s="15"/>
-      <c r="F42" s="11">
+      <c r="E42" s="14"/>
+      <c r="F42" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="11" t="s">
+      <c r="A43" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B43" s="11" t="s">
+      <c r="B43" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="C43" s="11" t="s">
+      <c r="C43" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="9">
         <f>VLOOKUP(C43,Overview!$G$2:$H$6,2,)</f>
         <v>4</v>
       </c>
-      <c r="E43" s="15"/>
-      <c r="F43" s="11">
+      <c r="E43" s="14"/>
+      <c r="F43" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="11" t="s">
+      <c r="A44" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="B44" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="C44" s="11" t="s">
+      <c r="C44" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D44" s="10">
+      <c r="D44" s="9">
         <f>VLOOKUP(C44,Overview!$G$2:$H$6,2,)</f>
         <v>4</v>
       </c>
-      <c r="E44" s="15"/>
-      <c r="F44" s="11">
+      <c r="E44" s="14"/>
+      <c r="F44" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="11" t="s">
+      <c r="A45" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B45" s="11" t="s">
+      <c r="B45" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C45" s="11" t="s">
+      <c r="C45" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D45" s="10">
+      <c r="D45" s="9">
         <f>VLOOKUP(C45,Overview!$G$2:$H$6,2,)</f>
         <v>4</v>
       </c>
-      <c r="E45" s="15"/>
-      <c r="F45" s="11">
+      <c r="E45" s="14"/>
+      <c r="F45" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="11" t="s">
+      <c r="A46" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="C46" s="11" t="s">
+      <c r="C46" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D46" s="10">
+      <c r="D46" s="9">
         <f>VLOOKUP(C46,Overview!$G$2:$H$6,2,)</f>
         <v>4</v>
       </c>
-      <c r="E46" s="15"/>
-      <c r="F46" s="11">
+      <c r="E46" s="14"/>
+      <c r="F46" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="11" t="s">
+      <c r="A47" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B47" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="C47" s="11" t="s">
+      <c r="C47" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D47" s="10">
+      <c r="D47" s="9">
         <f>VLOOKUP(C47,Overview!$G$2:$H$6,2,)</f>
         <v>4</v>
       </c>
-      <c r="E47" s="15"/>
-      <c r="F47" s="11">
+      <c r="E47" s="14"/>
+      <c r="F47" s="10">
         <v>20</v>
       </c>
     </row>

</xml_diff>